<commit_message>
Updated HOC values and guaranteed dispatch to align with real world dispatch.
</commit_message>
<xml_diff>
--- a/InputData/elec/HOC/HOC Hydro Opportunity Costs.xlsx
+++ b/InputData/elec/HOC/HOC Hydro Opportunity Costs.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\elec\HOC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\Mexico\Models\eps-mexico\InputData\elec\HOC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78F1369-79B6-4E42-BF97-B834263E8C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC702594-AB74-49FA-B686-EFE0CA7283EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30780" yWindow="2130" windowWidth="28245" windowHeight="12525" activeTab="1" xr2:uid="{8AA2DA0F-B30C-412A-A55D-748BA994FC4B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8AA2DA0F-B30C-412A-A55D-748BA994FC4B}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="HOC" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028" iterate="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -434,14 +434,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7655D3-EAD7-4119-BC82-55DAF4FF9FE5}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -457,27 +457,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -493,22 +493,22 @@
     <tabColor theme="3" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -517,18 +517,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -676,18 +676,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F0FCCF5-D8BA-4D2C-9680-AAB9C126C29B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BFBDA21-FFD2-4F6C-8952-40616E06B640}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F0FCCF5-D8BA-4D2C-9680-AAB9C126C29B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>